<commit_message>
indexing files, qdrant and app updated
</commit_message>
<xml_diff>
--- a/Data/Bachelors_programs.xlsx
+++ b/Data/Bachelors_programs.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mustafa Ansari\Downloads\Capestone_project_AI\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20C1F7F9-B644-4F64-B795-9233586E69E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DF916B2-B736-41AB-A5AB-9FA81C9DA353}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -324,9 +324,6 @@
     <t>Management, Decisions and Data Analytics | Constructor University</t>
   </si>
   <si>
-    <t>Fees_per_semester_euro</t>
-  </si>
-  <si>
     <t>On-campus_accommodation_fee_euro</t>
   </si>
   <si>
@@ -397,6 +394,9 @@
   </si>
   <si>
     <t>on_compus</t>
+  </si>
+  <si>
+    <t>Tuition_fees_per_semester_euro</t>
   </si>
 </sst>
 </file>
@@ -800,7 +800,7 @@
   <sheetData>
     <row r="1" spans="1:32" ht="51.5" thickBot="1">
       <c r="A1" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -827,13 +827,13 @@
         <v>6</v>
       </c>
       <c r="J1" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="K1" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="L1" s="6" t="s">
         <v>100</v>
-      </c>
-      <c r="L1" s="6" t="s">
-        <v>101</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>7</v>
@@ -878,7 +878,7 @@
         <v>20</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="AB1" s="1" t="s">
         <v>21</v>
@@ -896,7 +896,7 @@
     </row>
     <row r="2" spans="1:32" ht="114" thickBot="1">
       <c r="A2" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>25</v>
@@ -914,7 +914,7 @@
         <v>29</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H2" s="3">
         <v>3</v>
@@ -992,7 +992,7 @@
     </row>
     <row r="3" spans="1:32" ht="114" thickBot="1">
       <c r="A3" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>25</v>
@@ -1010,7 +1010,7 @@
         <v>29</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H3" s="3">
         <v>3</v>
@@ -1088,7 +1088,7 @@
     </row>
     <row r="4" spans="1:32" ht="139" thickBot="1">
       <c r="A4" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>25</v>
@@ -1106,7 +1106,7 @@
         <v>29</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H4" s="3">
         <v>3</v>
@@ -1184,7 +1184,7 @@
     </row>
     <row r="5" spans="1:32" ht="114" thickBot="1">
       <c r="A5" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>25</v>
@@ -1202,7 +1202,7 @@
         <v>29</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H5" s="3">
         <v>3</v>
@@ -1280,7 +1280,7 @@
     </row>
     <row r="6" spans="1:32" ht="114" thickBot="1">
       <c r="A6" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>25</v>
@@ -1298,7 +1298,7 @@
         <v>29</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H6" s="3">
         <v>3</v>
@@ -1376,7 +1376,7 @@
     </row>
     <row r="7" spans="1:32" ht="76.5" thickBot="1">
       <c r="A7" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>55</v>
@@ -1472,7 +1472,7 @@
     </row>
     <row r="8" spans="1:32" ht="76.5" thickBot="1">
       <c r="A8" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>55</v>
@@ -1481,7 +1481,7 @@
         <v>62</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>28</v>
@@ -1568,7 +1568,7 @@
     </row>
     <row r="9" spans="1:32" ht="114" thickBot="1">
       <c r="A9" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>55</v>
@@ -1586,7 +1586,7 @@
         <v>29</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H9" s="3">
         <v>3</v>
@@ -1664,7 +1664,7 @@
     </row>
     <row r="10" spans="1:32" ht="114" thickBot="1">
       <c r="A10" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>55</v>
@@ -1682,7 +1682,7 @@
         <v>29</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H10" s="3">
         <v>3</v>
@@ -1760,7 +1760,7 @@
     </row>
     <row r="11" spans="1:32" ht="114" thickBot="1">
       <c r="A11" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>55</v>
@@ -1778,7 +1778,7 @@
         <v>29</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H11" s="3">
         <v>3</v>
@@ -1856,7 +1856,7 @@
     </row>
     <row r="12" spans="1:32" ht="114" thickBot="1">
       <c r="A12" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>55</v>
@@ -1874,7 +1874,7 @@
         <v>29</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H12" s="3">
         <v>3</v>
@@ -1952,7 +1952,7 @@
     </row>
     <row r="13" spans="1:32" ht="114" thickBot="1">
       <c r="A13" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>55</v>
@@ -1970,7 +1970,7 @@
         <v>29</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H13" s="3">
         <v>3</v>
@@ -2048,7 +2048,7 @@
     </row>
     <row r="14" spans="1:32" ht="114" thickBot="1">
       <c r="A14" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>79</v>
@@ -2066,7 +2066,7 @@
         <v>82</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H14" s="3">
         <v>3</v>
@@ -2144,7 +2144,7 @@
     </row>
     <row r="15" spans="1:32" ht="114" thickBot="1">
       <c r="A15" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>79</v>
@@ -2162,7 +2162,7 @@
         <v>29</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H15" s="3">
         <v>3</v>
@@ -2240,7 +2240,7 @@
     </row>
     <row r="16" spans="1:32" ht="114" thickBot="1">
       <c r="A16" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>79</v>
@@ -2258,7 +2258,7 @@
         <v>29</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H16" s="3">
         <v>3</v>
@@ -2336,7 +2336,7 @@
     </row>
     <row r="17" spans="1:32" ht="114" thickBot="1">
       <c r="A17" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>79</v>
@@ -2354,7 +2354,7 @@
         <v>82</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H17" s="3">
         <v>3</v>
@@ -2432,7 +2432,7 @@
     </row>
     <row r="18" spans="1:32" ht="114" thickBot="1">
       <c r="A18" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>79</v>
@@ -2450,7 +2450,7 @@
         <v>82</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H18" s="3">
         <v>3</v>
@@ -2528,7 +2528,7 @@
     </row>
     <row r="19" spans="1:32" ht="114" thickBot="1">
       <c r="A19" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>79</v>
@@ -2546,7 +2546,7 @@
         <v>82</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H19" s="3">
         <v>3</v>

</xml_diff>